<commit_message>
decidindo arquivos e arrumando pre processamento
</commit_message>
<xml_diff>
--- a/LEM /LEM 2024.xlsx
+++ b/LEM /LEM 2024.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="0" windowWidth="19320" windowHeight="13020"/>
+    <workbookView xWindow="-120" yWindow="0" windowWidth="15600" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Plan1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
   <extLst>
@@ -188,7 +189,7 @@
     <t xml:space="preserve">                          EDUCAÇÃO</t>
   </si>
   <si>
-    <t>LEM - Levantamento estatístico Mensal/2024</t>
+    <t>LEM - Levantamento Estatístico Mensal/2024</t>
   </si>
 </sst>
 </file>
@@ -452,7 +453,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -499,15 +500,9 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1065,24 +1060,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="2"/>
       <c r="S1" s="3"/>
@@ -1094,22 +1089,22 @@
       <c r="Y1" s="3"/>
     </row>
     <row r="2" spans="1:25" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="42"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="6"/>
       <c r="S2" s="3"/>
@@ -1162,10 +1157,10 @@
       </c>
       <c r="N3" s="9"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="46" t="s">
+      <c r="P3" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="Q3" s="46"/>
+      <c r="Q3" s="44"/>
       <c r="R3" s="11"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
@@ -1176,51 +1171,55 @@
       <c r="Y3" s="3"/>
     </row>
     <row r="4" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="28" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="13">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="C4" s="13">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="D4" s="13">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E4" s="13">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="F4" s="13">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="G4" s="13">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="H4" s="13">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I4" s="13">
         <v>69</v>
       </c>
       <c r="J4" s="13">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="K4" s="13">
-        <v>68</v>
-      </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
+        <v>26</v>
+      </c>
+      <c r="L4" s="13">
+        <v>49</v>
+      </c>
+      <c r="M4" s="13">
+        <v>52</v>
+      </c>
       <c r="N4" s="14">
         <f>SUM(B4:M4)</f>
-        <v>625</v>
-      </c>
-      <c r="O4" s="28"/>
-      <c r="P4" s="34">
+        <v>701</v>
+      </c>
+      <c r="O4" s="26"/>
+      <c r="P4" s="32">
         <f>N21</f>
-        <v>1994</v>
-      </c>
-      <c r="Q4" s="35"/>
+        <v>0</v>
+      </c>
+      <c r="Q4" s="33"/>
       <c r="R4" s="18"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
@@ -1231,48 +1230,52 @@
       <c r="Y4" s="3"/>
     </row>
     <row r="5" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="28" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="13">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C5" s="13">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D5" s="13">
+        <v>50</v>
+      </c>
+      <c r="E5" s="13">
+        <v>52</v>
+      </c>
+      <c r="F5" s="13">
         <v>33</v>
       </c>
-      <c r="E5" s="13">
-        <v>26</v>
-      </c>
-      <c r="F5" s="13">
-        <v>29</v>
-      </c>
       <c r="G5" s="13">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="H5" s="13">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="I5" s="13">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="J5" s="13">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="K5" s="13">
-        <v>39</v>
-      </c>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
+        <v>7</v>
+      </c>
+      <c r="L5" s="13">
+        <v>30</v>
+      </c>
+      <c r="M5" s="13">
+        <v>28</v>
+      </c>
       <c r="N5" s="14">
-        <f t="shared" ref="N5:N20" si="0">SUM(B5:M5)</f>
-        <v>317</v>
-      </c>
-      <c r="O5" s="28"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="37"/>
+        <f t="shared" ref="N5:N29" si="0">SUM(B5:M5)</f>
+        <v>490</v>
+      </c>
+      <c r="O5" s="26"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="35"/>
       <c r="R5" s="18"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
@@ -1283,48 +1286,52 @@
       <c r="Y5" s="3"/>
     </row>
     <row r="6" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="28" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="13">
+        <v>24</v>
+      </c>
+      <c r="C6" s="13">
+        <v>21</v>
+      </c>
+      <c r="D6" s="13">
+        <v>15</v>
+      </c>
+      <c r="E6" s="13">
+        <v>19</v>
+      </c>
+      <c r="F6" s="13">
+        <v>25</v>
+      </c>
+      <c r="G6" s="13">
         <v>18</v>
       </c>
-      <c r="C6" s="13">
-        <v>20</v>
-      </c>
-      <c r="D6" s="13">
-        <v>23</v>
-      </c>
-      <c r="E6" s="13">
-        <v>9</v>
-      </c>
-      <c r="F6" s="13">
-        <v>19</v>
-      </c>
-      <c r="G6" s="13">
-        <v>13</v>
-      </c>
       <c r="H6" s="13">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="I6" s="13">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="J6" s="13">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K6" s="13">
         <v>16</v>
       </c>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
+      <c r="L6" s="13">
+        <v>17</v>
+      </c>
+      <c r="M6" s="13">
+        <v>12</v>
+      </c>
       <c r="N6" s="14">
         <f t="shared" si="0"/>
-        <v>152</v>
-      </c>
-      <c r="O6" s="28"/>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="37"/>
+        <v>222</v>
+      </c>
+      <c r="O6" s="26"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="35"/>
       <c r="R6" s="18"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
@@ -1335,48 +1342,52 @@
       <c r="Y6" s="3"/>
     </row>
     <row r="7" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="13">
+        <v>3</v>
+      </c>
+      <c r="C7" s="13">
+        <v>3</v>
+      </c>
+      <c r="D7" s="13">
+        <v>5</v>
+      </c>
+      <c r="E7" s="13">
+        <v>4</v>
+      </c>
+      <c r="F7" s="13">
+        <v>3</v>
+      </c>
+      <c r="G7" s="13">
         <v>2</v>
       </c>
-      <c r="C7" s="13">
-        <v>5</v>
-      </c>
-      <c r="D7" s="13">
+      <c r="H7" s="13">
+        <v>4</v>
+      </c>
+      <c r="I7" s="13">
         <v>7</v>
       </c>
-      <c r="E7" s="13">
+      <c r="J7" s="13">
         <v>6</v>
       </c>
-      <c r="F7" s="13">
-        <v>5</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="K7" s="13">
         <v>4</v>
       </c>
-      <c r="H7" s="13">
-        <v>7</v>
-      </c>
-      <c r="I7" s="13">
-        <v>4</v>
-      </c>
-      <c r="J7" s="13">
-        <v>11</v>
-      </c>
-      <c r="K7" s="13">
-        <v>7</v>
-      </c>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
+      <c r="L7" s="13">
+        <v>8</v>
+      </c>
+      <c r="M7" s="13">
+        <v>10</v>
+      </c>
       <c r="N7" s="14">
         <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-      <c r="O7" s="28"/>
-      <c r="P7" s="36"/>
-      <c r="Q7" s="37"/>
+        <v>59</v>
+      </c>
+      <c r="O7" s="26"/>
+      <c r="P7" s="34"/>
+      <c r="Q7" s="35"/>
       <c r="R7" s="18"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
@@ -1387,48 +1398,52 @@
       <c r="Y7" s="3"/>
     </row>
     <row r="8" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="28" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="13">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C8" s="13">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D8" s="13">
         <v>12</v>
       </c>
       <c r="E8" s="13">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F8" s="13">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G8" s="13">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H8" s="13">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I8" s="13">
         <v>9</v>
       </c>
       <c r="J8" s="13">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K8" s="13">
-        <v>12</v>
-      </c>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
+        <v>6</v>
+      </c>
+      <c r="L8" s="13">
+        <v>18</v>
+      </c>
+      <c r="M8" s="13">
+        <v>20</v>
+      </c>
       <c r="N8" s="14">
         <f t="shared" si="0"/>
-        <v>113</v>
-      </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="37"/>
+        <v>143</v>
+      </c>
+      <c r="O8" s="26"/>
+      <c r="P8" s="34"/>
+      <c r="Q8" s="35"/>
       <c r="R8" s="18"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3" t="s">
@@ -1441,48 +1456,52 @@
       <c r="Y8" s="3"/>
     </row>
     <row r="9" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="28" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="13">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C9" s="13">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="D9" s="13">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E9" s="13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" s="13">
+        <v>7</v>
+      </c>
+      <c r="G9" s="13">
+        <v>4</v>
+      </c>
+      <c r="H9" s="13">
+        <v>5</v>
+      </c>
+      <c r="I9" s="13">
+        <v>11</v>
+      </c>
+      <c r="J9" s="13">
+        <v>23</v>
+      </c>
+      <c r="K9" s="13">
+        <v>7</v>
+      </c>
+      <c r="L9" s="13">
         <v>10</v>
       </c>
-      <c r="G9" s="13">
-        <v>27</v>
-      </c>
-      <c r="H9" s="13">
-        <v>16</v>
-      </c>
-      <c r="I9" s="13">
-        <v>28</v>
-      </c>
-      <c r="J9" s="13">
-        <v>29</v>
-      </c>
-      <c r="K9" s="13">
-        <v>32</v>
-      </c>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
+      <c r="M9" s="13">
+        <v>25</v>
+      </c>
       <c r="N9" s="14">
         <f t="shared" si="0"/>
-        <v>229</v>
-      </c>
-      <c r="O9" s="28"/>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="37"/>
+        <v>137</v>
+      </c>
+      <c r="O9" s="26"/>
+      <c r="P9" s="34"/>
+      <c r="Q9" s="35"/>
       <c r="R9" s="18"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
@@ -1493,20 +1512,20 @@
       <c r="Y9" s="3"/>
     </row>
     <row r="10" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="28" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="13">
+        <v>20</v>
+      </c>
+      <c r="C10" s="13">
+        <v>19</v>
+      </c>
+      <c r="D10" s="13">
         <v>7</v>
       </c>
-      <c r="C10" s="13">
-        <v>23</v>
-      </c>
-      <c r="D10" s="13">
-        <v>14</v>
-      </c>
       <c r="E10" s="13">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F10" s="13">
         <v>7</v>
@@ -1515,26 +1534,30 @@
         <v>8</v>
       </c>
       <c r="H10" s="13">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="I10" s="13">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J10" s="13">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="K10" s="13">
-        <v>18</v>
-      </c>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
+        <v>15</v>
+      </c>
+      <c r="L10" s="13">
+        <v>9</v>
+      </c>
+      <c r="M10" s="13">
+        <v>13</v>
+      </c>
       <c r="N10" s="14">
         <f t="shared" si="0"/>
-        <v>135</v>
-      </c>
-      <c r="O10" s="28"/>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="37"/>
+        <v>140</v>
+      </c>
+      <c r="O10" s="26"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="35"/>
       <c r="R10" s="18"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
@@ -1545,48 +1568,52 @@
       <c r="Y10" s="3"/>
     </row>
     <row r="11" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="28" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="13">
         <v>1</v>
       </c>
       <c r="C11" s="13">
+        <v>0</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
         <v>1</v>
       </c>
-      <c r="D11" s="13">
+      <c r="F11" s="13">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
         <v>1</v>
       </c>
-      <c r="E11" s="13">
-        <v>0</v>
-      </c>
-      <c r="F11" s="13">
-        <v>2</v>
-      </c>
-      <c r="G11" s="13">
-        <v>2</v>
-      </c>
       <c r="H11" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J11" s="13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K11" s="13">
-        <v>3</v>
-      </c>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="L11" s="13">
+        <v>0</v>
+      </c>
+      <c r="M11" s="13">
+        <v>0</v>
+      </c>
       <c r="N11" s="14">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="O11" s="28"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="37"/>
+        <v>7</v>
+      </c>
+      <c r="O11" s="26"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="35"/>
       <c r="R11" s="18"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
@@ -1597,42 +1624,52 @@
       <c r="Y11" s="3"/>
     </row>
     <row r="12" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
+      <c r="B12" s="13">
+        <v>3</v>
+      </c>
+      <c r="C12" s="13">
+        <v>4</v>
+      </c>
+      <c r="D12" s="13">
+        <v>5</v>
+      </c>
       <c r="E12" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" s="13">
+        <v>7</v>
+      </c>
+      <c r="G12" s="13">
         <v>2</v>
       </c>
-      <c r="G12" s="13">
-        <v>1</v>
-      </c>
       <c r="H12" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" s="13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J12" s="13">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K12" s="13">
-        <v>2</v>
-      </c>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
+        <v>4</v>
+      </c>
+      <c r="L12" s="13">
+        <v>8</v>
+      </c>
+      <c r="M12" s="13">
+        <v>10</v>
+      </c>
       <c r="N12" s="14">
         <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="O12" s="28"/>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="37"/>
+        <v>64</v>
+      </c>
+      <c r="O12" s="26"/>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="35"/>
       <c r="R12" s="18"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
@@ -1643,46 +1680,52 @@
       <c r="Y12" s="3"/>
     </row>
     <row r="13" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="28" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C13" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D13" s="13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E13" s="13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F13" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G13" s="13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13" s="13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I13" s="13">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J13" s="13">
-        <v>0</v>
-      </c>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
+        <v>6</v>
+      </c>
+      <c r="K13" s="13">
+        <v>4</v>
+      </c>
+      <c r="L13" s="13">
+        <v>8</v>
+      </c>
+      <c r="M13" s="13">
+        <v>10</v>
+      </c>
       <c r="N13" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O13" s="28"/>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="37"/>
+        <v>59</v>
+      </c>
+      <c r="O13" s="26"/>
+      <c r="P13" s="34"/>
+      <c r="Q13" s="35"/>
       <c r="R13" s="18"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
@@ -1693,46 +1736,52 @@
       <c r="Y13" s="3"/>
     </row>
     <row r="14" spans="1:25" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="13"/>
+      <c r="B14" s="13">
+        <v>5</v>
+      </c>
       <c r="C14" s="13">
+        <v>5</v>
+      </c>
+      <c r="D14" s="13">
         <v>12</v>
       </c>
-      <c r="D14" s="13">
-        <v>8</v>
-      </c>
       <c r="E14" s="13">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F14" s="13">
         <v>9</v>
       </c>
       <c r="G14" s="13">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="H14" s="13">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I14" s="13">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J14" s="13">
+        <v>12</v>
+      </c>
+      <c r="K14" s="13">
+        <v>10</v>
+      </c>
+      <c r="L14" s="13">
+        <v>12</v>
+      </c>
+      <c r="M14" s="13">
         <v>11</v>
       </c>
-      <c r="K14" s="13">
-        <v>12</v>
-      </c>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
       <c r="N14" s="14">
         <f t="shared" si="0"/>
-        <v>78</v>
-      </c>
-      <c r="O14" s="28"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="37"/>
+        <v>118</v>
+      </c>
+      <c r="O14" s="26"/>
+      <c r="P14" s="34"/>
+      <c r="Q14" s="35"/>
       <c r="R14" s="18"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
@@ -1743,48 +1792,52 @@
       <c r="Y14" s="3"/>
     </row>
     <row r="15" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="28" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C15" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="13">
+        <v>5</v>
+      </c>
+      <c r="E15" s="13">
         <v>4</v>
       </c>
-      <c r="E15" s="13">
-        <v>0</v>
-      </c>
       <c r="F15" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15" s="13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" s="13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I15" s="13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J15" s="13">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K15" s="13">
-        <v>1</v>
-      </c>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
+        <v>4</v>
+      </c>
+      <c r="L15" s="13">
+        <v>8</v>
+      </c>
+      <c r="M15" s="13">
+        <v>0</v>
+      </c>
       <c r="N15" s="14">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="O15" s="28"/>
-      <c r="P15" s="36"/>
-      <c r="Q15" s="37"/>
+        <v>49</v>
+      </c>
+      <c r="O15" s="26"/>
+      <c r="P15" s="34"/>
+      <c r="Q15" s="35"/>
       <c r="R15" s="18"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
@@ -1795,48 +1848,52 @@
       <c r="Y15" s="3"/>
     </row>
     <row r="16" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="28" t="s">
         <v>26</v>
       </c>
       <c r="B16" s="13">
+        <v>0</v>
+      </c>
+      <c r="C16" s="13">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13">
+        <v>10</v>
+      </c>
+      <c r="E16" s="13">
         <v>2</v>
       </c>
-      <c r="C16" s="13">
-        <v>4</v>
-      </c>
-      <c r="D16" s="13">
-        <v>4</v>
-      </c>
-      <c r="E16" s="13">
-        <v>5</v>
-      </c>
       <c r="F16" s="13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G16" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I16" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J16" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" s="13">
-        <v>2</v>
-      </c>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="L16" s="13">
+        <v>0</v>
+      </c>
+      <c r="M16" s="13">
+        <v>0</v>
+      </c>
       <c r="N16" s="14">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="O16" s="17"/>
-      <c r="P16" s="36"/>
-      <c r="Q16" s="37"/>
+      <c r="P16" s="34"/>
+      <c r="Q16" s="35"/>
       <c r="R16" s="18"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
@@ -1847,48 +1904,52 @@
       <c r="Y16" s="3"/>
     </row>
     <row r="17" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="28" t="s">
         <v>27</v>
       </c>
       <c r="B17" s="13">
         <v>0</v>
       </c>
       <c r="C17" s="13">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13">
+        <v>0</v>
+      </c>
+      <c r="E17" s="13">
+        <v>0</v>
+      </c>
+      <c r="F17" s="13">
+        <v>0</v>
+      </c>
+      <c r="G17" s="13">
+        <v>1</v>
+      </c>
+      <c r="H17" s="13">
+        <v>4</v>
+      </c>
+      <c r="I17" s="13">
+        <v>0</v>
+      </c>
+      <c r="J17" s="13">
+        <v>0</v>
+      </c>
+      <c r="K17" s="13">
         <v>2</v>
       </c>
-      <c r="D17" s="13">
-        <v>1</v>
-      </c>
-      <c r="E17" s="13">
-        <v>0</v>
-      </c>
-      <c r="F17" s="13">
-        <v>1</v>
-      </c>
-      <c r="G17" s="13">
-        <v>6</v>
-      </c>
-      <c r="H17" s="13">
-        <v>0</v>
-      </c>
-      <c r="I17" s="13">
-        <v>3</v>
-      </c>
-      <c r="J17" s="13">
-        <v>0</v>
-      </c>
-      <c r="K17" s="13">
-        <v>6</v>
-      </c>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
+      <c r="L17" s="13">
+        <v>0</v>
+      </c>
+      <c r="M17" s="13">
+        <v>0</v>
+      </c>
       <c r="N17" s="14">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="O17" s="17"/>
-      <c r="P17" s="36"/>
-      <c r="Q17" s="37"/>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="35"/>
       <c r="R17" s="18"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
@@ -1899,21 +1960,23 @@
       <c r="Y17" s="3"/>
     </row>
     <row r="18" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="28" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="13">
-        <v>1</v>
-      </c>
-      <c r="C18" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="C18" s="13">
+        <v>0</v>
+      </c>
       <c r="D18" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" s="13">
         <v>1</v>
       </c>
       <c r="F18" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="13">
         <v>0</v>
@@ -1922,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J18" s="13">
         <v>0</v>
@@ -1930,15 +1993,19 @@
       <c r="K18" s="13">
         <v>1</v>
       </c>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
+      <c r="L18" s="13">
+        <v>0</v>
+      </c>
+      <c r="M18" s="13">
+        <v>0</v>
+      </c>
       <c r="N18" s="14">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O18" s="17"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="37"/>
+      <c r="P18" s="34"/>
+      <c r="Q18" s="35"/>
       <c r="R18" s="18"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
@@ -1951,48 +2018,52 @@
       <c r="Y18" s="3"/>
     </row>
     <row r="19" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="28" t="s">
         <v>29</v>
       </c>
       <c r="B19" s="13">
+        <v>20</v>
+      </c>
+      <c r="C19" s="13">
+        <v>20</v>
+      </c>
+      <c r="D19" s="13">
+        <v>20</v>
+      </c>
+      <c r="E19" s="13">
+        <v>19</v>
+      </c>
+      <c r="F19" s="13">
         <v>18</v>
-      </c>
-      <c r="C19" s="13">
-        <v>19</v>
-      </c>
-      <c r="D19" s="13">
-        <v>18</v>
-      </c>
-      <c r="E19" s="13">
-        <v>14</v>
-      </c>
-      <c r="F19" s="13">
-        <v>11</v>
       </c>
       <c r="G19" s="13">
         <v>17</v>
       </c>
       <c r="H19" s="13">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I19" s="13">
         <v>18</v>
       </c>
       <c r="J19" s="13">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K19" s="13">
-        <v>19</v>
-      </c>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="L19" s="13">
+        <v>17</v>
+      </c>
+      <c r="M19" s="13">
+        <v>18</v>
+      </c>
       <c r="N19" s="14">
         <f t="shared" si="0"/>
-        <v>161</v>
+        <v>220</v>
       </c>
       <c r="O19" s="17"/>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="37"/>
+      <c r="P19" s="34"/>
+      <c r="Q19" s="35"/>
       <c r="R19" s="18"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
@@ -2003,48 +2074,52 @@
       <c r="Y19" s="3"/>
     </row>
     <row r="20" spans="1:29" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="28" t="s">
         <v>30</v>
       </c>
       <c r="B20" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" s="13">
         <v>1</v>
       </c>
       <c r="F20" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H20" s="13">
+        <v>0</v>
+      </c>
+      <c r="I20" s="13">
         <v>5</v>
       </c>
-      <c r="I20" s="13">
-        <v>2</v>
-      </c>
       <c r="J20" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K20" s="13">
-        <v>12</v>
-      </c>
-      <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="L20" s="13">
+        <v>0</v>
+      </c>
+      <c r="M20" s="13">
+        <v>0</v>
+      </c>
       <c r="N20" s="14">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="O20" s="17"/>
-      <c r="P20" s="38"/>
-      <c r="Q20" s="39"/>
+      <c r="P20" s="36"/>
+      <c r="Q20" s="37"/>
       <c r="R20" s="18"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
@@ -2070,15 +2145,15 @@
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
-      <c r="N21" s="27">
-        <f>SUM(N4:N20)</f>
-        <v>1994</v>
+      <c r="N21" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="O21" s="17"/>
-      <c r="P21" s="47" t="s">
+      <c r="P21" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="Q21" s="47"/>
+      <c r="Q21" s="45"/>
       <c r="R21" s="18"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
@@ -2089,37 +2164,55 @@
       <c r="Y21" s="3"/>
     </row>
     <row r="22" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
+      <c r="B22" s="19">
+        <v>2</v>
+      </c>
+      <c r="C22" s="19">
+        <v>2</v>
+      </c>
+      <c r="D22" s="19">
+        <v>0</v>
+      </c>
+      <c r="E22" s="19">
+        <v>0</v>
+      </c>
+      <c r="F22" s="19">
+        <v>0</v>
+      </c>
+      <c r="G22" s="19">
+        <v>0</v>
+      </c>
+      <c r="H22" s="19">
+        <v>0</v>
+      </c>
       <c r="I22" s="19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" s="19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="19">
         <v>0</v>
       </c>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="20">
-        <f>SUM(B22:M22)</f>
-        <v>2</v>
-      </c>
-      <c r="O22" s="28"/>
-      <c r="P22" s="34">
+      <c r="L22" s="19">
+        <v>0</v>
+      </c>
+      <c r="M22" s="19">
+        <v>0</v>
+      </c>
+      <c r="N22" s="14">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="O22" s="26"/>
+      <c r="P22" s="32">
         <f>N26</f>
-        <v>10</v>
-      </c>
-      <c r="Q22" s="35"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="33"/>
       <c r="R22" s="18"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
@@ -2129,37 +2222,53 @@
       <c r="X22" s="3"/>
       <c r="Y22" s="3"/>
     </row>
-    <row r="23" spans="1:29" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="31" t="s">
+    <row r="23" spans="1:29" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="19"/>
+      <c r="B23" s="19">
+        <v>3</v>
+      </c>
       <c r="C23" s="19">
+        <v>0</v>
+      </c>
+      <c r="D23" s="19">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19">
+        <v>0</v>
+      </c>
+      <c r="F23" s="19">
+        <v>0</v>
+      </c>
+      <c r="G23" s="19">
+        <v>0</v>
+      </c>
+      <c r="H23" s="19">
+        <v>0</v>
+      </c>
+      <c r="I23" s="19">
+        <v>0</v>
+      </c>
+      <c r="J23" s="19">
         <v>1</v>
       </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19">
-        <v>1</v>
-      </c>
-      <c r="J23" s="19">
-        <v>2</v>
-      </c>
       <c r="K23" s="19">
+        <v>0</v>
+      </c>
+      <c r="L23" s="19">
+        <v>0</v>
+      </c>
+      <c r="M23" s="19">
+        <v>0</v>
+      </c>
+      <c r="N23" s="14">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="20">
-        <f t="shared" ref="N23:N25" si="1">SUM(B23:M23)</f>
-        <v>8</v>
-      </c>
-      <c r="O23" s="28"/>
-      <c r="P23" s="36"/>
-      <c r="Q23" s="37"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="34"/>
+      <c r="Q23" s="35"/>
       <c r="R23" s="18"/>
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
@@ -2173,33 +2282,53 @@
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
     </row>
-    <row r="24" spans="1:29" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:29" s="21" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
+      <c r="B24" s="13">
+        <v>7</v>
+      </c>
+      <c r="C24" s="13">
+        <v>13</v>
+      </c>
+      <c r="D24" s="13">
+        <v>10</v>
+      </c>
+      <c r="E24" s="13">
+        <v>15</v>
+      </c>
+      <c r="F24" s="13">
+        <v>6</v>
+      </c>
+      <c r="G24" s="13">
+        <v>9</v>
+      </c>
+      <c r="H24" s="13">
+        <v>5</v>
+      </c>
+      <c r="I24" s="13">
+        <v>9</v>
+      </c>
       <c r="J24" s="13">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K24" s="13">
-        <v>0</v>
-      </c>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="20">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O24" s="28"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="37"/>
+        <v>6</v>
+      </c>
+      <c r="L24" s="13">
+        <v>6</v>
+      </c>
+      <c r="M24" s="13">
+        <v>0</v>
+      </c>
+      <c r="N24" s="14">
+        <f t="shared" si="0"/>
+        <v>94</v>
+      </c>
+      <c r="O24" s="26"/>
+      <c r="P24" s="34"/>
+      <c r="Q24" s="35"/>
       <c r="R24" s="18"/>
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
@@ -2214,32 +2343,52 @@
       <c r="AC24" s="4"/>
     </row>
     <row r="25" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23">
-        <v>0</v>
-      </c>
-      <c r="K25" s="23">
-        <v>0</v>
-      </c>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
+      <c r="B25" s="13">
+        <v>7</v>
+      </c>
+      <c r="C25" s="13">
+        <v>12</v>
+      </c>
+      <c r="D25" s="13">
+        <v>13</v>
+      </c>
+      <c r="E25" s="13">
+        <v>15</v>
+      </c>
+      <c r="F25" s="13">
+        <v>6</v>
+      </c>
+      <c r="G25" s="13">
+        <v>7</v>
+      </c>
+      <c r="H25" s="13">
+        <v>8</v>
+      </c>
+      <c r="I25" s="13">
+        <v>10</v>
+      </c>
+      <c r="J25" s="13">
+        <v>8</v>
+      </c>
+      <c r="K25" s="13">
+        <v>7</v>
+      </c>
+      <c r="L25" s="13">
+        <v>6</v>
+      </c>
+      <c r="M25" s="22">
+        <v>4</v>
+      </c>
       <c r="N25" s="14">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>103</v>
       </c>
       <c r="O25" s="17"/>
-      <c r="P25" s="38"/>
-      <c r="Q25" s="39"/>
+      <c r="P25" s="36"/>
+      <c r="Q25" s="37"/>
       <c r="R25" s="18"/>
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
@@ -2265,15 +2414,15 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
       <c r="M26" s="8"/>
-      <c r="N26" s="27">
-        <f>SUM(N22:N25)</f>
-        <v>10</v>
+      <c r="N26" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="O26" s="17"/>
-      <c r="P26" s="47" t="s">
+      <c r="P26" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="Q26" s="47"/>
+      <c r="Q26" s="45"/>
       <c r="R26" s="18"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
@@ -2288,45 +2437,51 @@
         <v>39</v>
       </c>
       <c r="B27" s="13">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C27" s="13">
+        <v>37</v>
+      </c>
+      <c r="D27" s="13">
+        <v>33</v>
+      </c>
+      <c r="E27" s="13">
+        <v>39</v>
+      </c>
+      <c r="F27" s="13">
         <v>23</v>
       </c>
-      <c r="D27" s="13">
+      <c r="G27" s="13">
+        <v>25</v>
+      </c>
+      <c r="H27" s="13">
+        <v>35</v>
+      </c>
+      <c r="I27" s="13">
+        <v>29</v>
+      </c>
+      <c r="J27" s="13">
+        <v>18</v>
+      </c>
+      <c r="K27" s="13">
         <v>15</v>
       </c>
-      <c r="E27" s="13">
-        <v>18</v>
-      </c>
-      <c r="F27" s="13">
-        <v>16</v>
-      </c>
-      <c r="G27" s="13">
-        <v>14</v>
-      </c>
-      <c r="H27" s="13">
-        <v>18</v>
-      </c>
-      <c r="I27" s="13">
-        <v>20</v>
-      </c>
-      <c r="J27" s="13">
-        <v>21</v>
-      </c>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="24">
-        <f>SUM(B27:M27)</f>
-        <v>165</v>
+      <c r="L27" s="13">
+        <v>29</v>
+      </c>
+      <c r="M27" s="13">
+        <v>36</v>
+      </c>
+      <c r="N27" s="14">
+        <f t="shared" si="0"/>
+        <v>358</v>
       </c>
       <c r="O27" s="15"/>
-      <c r="P27" s="48">
+      <c r="P27" s="46">
         <f>N30</f>
-        <v>352</v>
-      </c>
-      <c r="Q27" s="48"/>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="46"/>
       <c r="R27" s="16"/>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
@@ -2344,39 +2499,45 @@
         <v>20</v>
       </c>
       <c r="C28" s="13">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D28" s="13">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E28" s="13">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F28" s="13">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G28" s="13">
         <v>20</v>
       </c>
       <c r="H28" s="13">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I28" s="13">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="J28" s="13">
+        <v>19</v>
+      </c>
+      <c r="K28" s="13">
         <v>20</v>
       </c>
-      <c r="K28" s="13"/>
-      <c r="L28" s="13"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="24">
-        <f t="shared" ref="N28:N29" si="2">SUM(B28:M28)</f>
-        <v>185</v>
+      <c r="L28" s="13">
+        <v>16</v>
+      </c>
+      <c r="M28" s="13">
+        <v>17</v>
+      </c>
+      <c r="N28" s="14">
+        <f t="shared" si="0"/>
+        <v>206</v>
       </c>
       <c r="O28" s="15"/>
-      <c r="P28" s="48"/>
-      <c r="Q28" s="48"/>
+      <c r="P28" s="46"/>
+      <c r="Q28" s="46"/>
       <c r="R28" s="16"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -2387,23 +2548,23 @@
       <c r="Y28" s="3"/>
     </row>
     <row r="29" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="23" t="s">
         <v>41</v>
       </c>
       <c r="B29" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C29" s="13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D29" s="13">
         <v>0</v>
       </c>
       <c r="E29" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="13">
         <v>0</v>
@@ -2412,21 +2573,27 @@
         <v>0</v>
       </c>
       <c r="I29" s="13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J29" s="13">
-        <v>2</v>
-      </c>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="24">
-        <f t="shared" si="2"/>
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="K29" s="13">
+        <v>0</v>
+      </c>
+      <c r="L29" s="13">
+        <v>0</v>
+      </c>
+      <c r="M29" s="13">
+        <v>1</v>
+      </c>
+      <c r="N29" s="14">
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="O29" s="15"/>
-      <c r="P29" s="48"/>
-      <c r="Q29" s="48"/>
+      <c r="P29" s="46"/>
+      <c r="Q29" s="46"/>
       <c r="R29" s="16"/>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
@@ -2437,30 +2604,27 @@
       <c r="Y29" s="3"/>
     </row>
     <row r="30" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="26" t="s">
+      <c r="A30" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27">
-        <f>SUM(N27:N29)</f>
-        <v>352</v>
-      </c>
-      <c r="O30" s="49"/>
-      <c r="P30" s="50" t="s">
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="25"/>
+      <c r="M30" s="25"/>
+      <c r="N30" s="25"/>
+      <c r="O30" s="47"/>
+      <c r="P30" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="Q30" s="50"/>
+      <c r="Q30" s="48"/>
       <c r="R30" s="18"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
@@ -2471,7 +2635,7 @@
       <c r="Y30" s="3"/>
     </row>
     <row r="31" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="31" t="s">
         <v>43</v>
       </c>
       <c r="B31" s="13"/>
@@ -2487,12 +2651,12 @@
       <c r="L31" s="13"/>
       <c r="M31" s="13"/>
       <c r="N31" s="14"/>
-      <c r="O31" s="49"/>
-      <c r="P31" s="34">
+      <c r="O31" s="47"/>
+      <c r="P31" s="32">
         <f>N44</f>
         <v>0</v>
       </c>
-      <c r="Q31" s="35"/>
+      <c r="Q31" s="33"/>
       <c r="R31" s="18"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
@@ -2503,30 +2667,49 @@
       <c r="Y31" s="3"/>
     </row>
     <row r="32" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
+      <c r="B32" s="13">
+        <v>1</v>
+      </c>
+      <c r="C32" s="13">
+        <v>0</v>
+      </c>
+      <c r="D32" s="13">
+        <v>0</v>
+      </c>
+      <c r="E32" s="13">
+        <v>0</v>
+      </c>
+      <c r="F32" s="13">
+        <v>0</v>
+      </c>
+      <c r="G32" s="13">
+        <v>0</v>
+      </c>
+      <c r="H32" s="13">
+        <v>0</v>
+      </c>
+      <c r="I32" s="13">
+        <v>2</v>
+      </c>
+      <c r="J32" s="13">
+        <v>1</v>
+      </c>
       <c r="K32" s="13">
-        <v>1</v>
-      </c>
-      <c r="L32" s="13"/>
-      <c r="M32" s="13"/>
-      <c r="N32" s="14">
-        <f>SUM(B32:M32)</f>
-        <v>1</v>
-      </c>
-      <c r="O32" s="49"/>
-      <c r="P32" s="36"/>
-      <c r="Q32" s="37"/>
+        <v>0</v>
+      </c>
+      <c r="L32" s="13">
+        <v>0</v>
+      </c>
+      <c r="M32" s="13">
+        <v>0</v>
+      </c>
+      <c r="N32" s="14"/>
+      <c r="O32" s="47"/>
+      <c r="P32" s="34"/>
+      <c r="Q32" s="35"/>
       <c r="R32" s="18"/>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
@@ -2537,28 +2720,47 @@
       <c r="Y32" s="3"/>
     </row>
     <row r="33" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="31" t="s">
         <v>45</v>
       </c>
       <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
-      <c r="N33" s="14">
-        <f t="shared" ref="N33:N43" si="3">SUM(B33:M33)</f>
-        <v>0</v>
-      </c>
-      <c r="O33" s="49"/>
-      <c r="P33" s="36"/>
-      <c r="Q33" s="37"/>
+      <c r="C33" s="13">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0</v>
+      </c>
+      <c r="E33" s="13">
+        <v>0</v>
+      </c>
+      <c r="F33" s="13">
+        <v>1</v>
+      </c>
+      <c r="G33" s="13">
+        <v>0</v>
+      </c>
+      <c r="H33" s="13">
+        <v>2</v>
+      </c>
+      <c r="I33" s="13">
+        <v>0</v>
+      </c>
+      <c r="J33" s="13">
+        <v>0</v>
+      </c>
+      <c r="K33" s="13">
+        <v>0</v>
+      </c>
+      <c r="L33" s="13">
+        <v>0</v>
+      </c>
+      <c r="M33" s="13">
+        <v>0</v>
+      </c>
+      <c r="N33" s="14"/>
+      <c r="O33" s="47"/>
+      <c r="P33" s="34"/>
+      <c r="Q33" s="35"/>
       <c r="R33" s="18"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
@@ -2569,7 +2771,7 @@
       <c r="Y33" s="3"/>
     </row>
     <row r="34" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="33" t="s">
+      <c r="A34" s="31" t="s">
         <v>46</v>
       </c>
       <c r="B34" s="13"/>
@@ -2584,13 +2786,10 @@
       <c r="K34" s="13"/>
       <c r="L34" s="13"/>
       <c r="M34" s="13"/>
-      <c r="N34" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O34" s="49"/>
-      <c r="P34" s="36"/>
-      <c r="Q34" s="37"/>
+      <c r="N34" s="14"/>
+      <c r="O34" s="47"/>
+      <c r="P34" s="34"/>
+      <c r="Q34" s="35"/>
       <c r="R34" s="18"/>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
@@ -2601,40 +2800,49 @@
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="13"/>
+      <c r="B35" s="13">
+        <v>2</v>
+      </c>
       <c r="C35" s="13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D35" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E35" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="13">
-        <v>3</v>
-      </c>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="G35" s="13">
+        <v>0</v>
+      </c>
+      <c r="H35" s="13">
+        <v>0</v>
+      </c>
       <c r="I35" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" s="13">
         <v>1</v>
       </c>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="14">
-        <f t="shared" si="3"/>
-        <v>12</v>
-      </c>
-      <c r="O35" s="49"/>
-      <c r="P35" s="36"/>
-      <c r="Q35" s="37"/>
+      <c r="K35" s="13">
+        <v>0</v>
+      </c>
+      <c r="L35" s="13">
+        <v>2</v>
+      </c>
+      <c r="M35" s="13">
+        <v>0</v>
+      </c>
+      <c r="N35" s="14"/>
+      <c r="O35" s="47"/>
+      <c r="P35" s="34"/>
+      <c r="Q35" s="35"/>
       <c r="R35" s="18"/>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
@@ -2645,28 +2853,49 @@
       <c r="Y35" s="3"/>
     </row>
     <row r="36" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="33" t="s">
+      <c r="A36" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="13"/>
-      <c r="M36" s="13"/>
-      <c r="N36" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O36" s="49"/>
-      <c r="P36" s="36"/>
-      <c r="Q36" s="37"/>
+      <c r="B36" s="13">
+        <v>0</v>
+      </c>
+      <c r="C36" s="13">
+        <v>0</v>
+      </c>
+      <c r="D36" s="13">
+        <v>0</v>
+      </c>
+      <c r="E36" s="13">
+        <v>0</v>
+      </c>
+      <c r="F36" s="13">
+        <v>0</v>
+      </c>
+      <c r="G36" s="13">
+        <v>0</v>
+      </c>
+      <c r="H36" s="13">
+        <v>0</v>
+      </c>
+      <c r="I36" s="13">
+        <v>0</v>
+      </c>
+      <c r="J36" s="13">
+        <v>0</v>
+      </c>
+      <c r="K36" s="13">
+        <v>0</v>
+      </c>
+      <c r="L36" s="13">
+        <v>0</v>
+      </c>
+      <c r="M36" s="13">
+        <v>0</v>
+      </c>
+      <c r="N36" s="14"/>
+      <c r="O36" s="47"/>
+      <c r="P36" s="34"/>
+      <c r="Q36" s="35"/>
       <c r="R36" s="18"/>
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
@@ -2677,7 +2906,7 @@
       <c r="Y36" s="3"/>
     </row>
     <row r="37" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="33" t="s">
+      <c r="A37" s="31" t="s">
         <v>47</v>
       </c>
       <c r="B37" s="13"/>
@@ -2692,13 +2921,10 @@
       <c r="K37" s="13"/>
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
-      <c r="N37" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O37" s="49"/>
-      <c r="P37" s="36"/>
-      <c r="Q37" s="37"/>
+      <c r="N37" s="14"/>
+      <c r="O37" s="47"/>
+      <c r="P37" s="34"/>
+      <c r="Q37" s="35"/>
       <c r="R37" s="18"/>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
@@ -2709,32 +2935,49 @@
       <c r="Y37" s="3"/>
     </row>
     <row r="38" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="32" t="s">
+      <c r="A38" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23">
+      <c r="B38" s="22">
         <v>2</v>
       </c>
-      <c r="H38" s="23"/>
-      <c r="I38" s="23">
-        <v>2</v>
-      </c>
-      <c r="J38" s="23"/>
-      <c r="K38" s="23"/>
-      <c r="L38" s="23"/>
-      <c r="M38" s="23"/>
-      <c r="N38" s="14">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="O38" s="49"/>
-      <c r="P38" s="36"/>
-      <c r="Q38" s="37"/>
+      <c r="C38" s="22">
+        <v>1</v>
+      </c>
+      <c r="D38" s="22">
+        <v>1</v>
+      </c>
+      <c r="E38" s="22">
+        <v>0</v>
+      </c>
+      <c r="F38" s="22">
+        <v>0</v>
+      </c>
+      <c r="G38" s="22">
+        <v>0</v>
+      </c>
+      <c r="H38" s="22">
+        <v>0</v>
+      </c>
+      <c r="I38" s="22">
+        <v>0</v>
+      </c>
+      <c r="J38" s="22">
+        <v>0</v>
+      </c>
+      <c r="K38" s="22">
+        <v>0</v>
+      </c>
+      <c r="L38" s="22">
+        <v>0</v>
+      </c>
+      <c r="M38" s="22">
+        <v>0</v>
+      </c>
+      <c r="N38" s="14"/>
+      <c r="O38" s="47"/>
+      <c r="P38" s="34"/>
+      <c r="Q38" s="35"/>
       <c r="R38" s="18"/>
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
@@ -2745,28 +2988,49 @@
       <c r="Y38" s="3"/>
     </row>
     <row r="39" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="33" t="s">
+      <c r="A39" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="13"/>
-      <c r="N39" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O39" s="28"/>
-      <c r="P39" s="36"/>
-      <c r="Q39" s="37"/>
+      <c r="B39" s="13">
+        <v>0</v>
+      </c>
+      <c r="C39" s="13">
+        <v>0</v>
+      </c>
+      <c r="D39" s="13">
+        <v>0</v>
+      </c>
+      <c r="E39" s="13">
+        <v>0</v>
+      </c>
+      <c r="F39" s="13">
+        <v>0</v>
+      </c>
+      <c r="G39" s="13">
+        <v>0</v>
+      </c>
+      <c r="H39" s="13">
+        <v>0</v>
+      </c>
+      <c r="I39" s="13">
+        <v>0</v>
+      </c>
+      <c r="J39" s="13">
+        <v>0</v>
+      </c>
+      <c r="K39" s="13">
+        <v>0</v>
+      </c>
+      <c r="L39" s="13">
+        <v>0</v>
+      </c>
+      <c r="M39" s="13">
+        <v>0</v>
+      </c>
+      <c r="N39" s="14"/>
+      <c r="O39" s="26"/>
+      <c r="P39" s="34"/>
+      <c r="Q39" s="35"/>
       <c r="R39" s="18"/>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
@@ -2777,7 +3041,7 @@
       <c r="Y39" s="3"/>
     </row>
     <row r="40" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="30" t="s">
+      <c r="A40" s="28" t="s">
         <v>48</v>
       </c>
       <c r="B40" s="13"/>
@@ -2792,13 +3056,10 @@
       <c r="K40" s="13"/>
       <c r="L40" s="13"/>
       <c r="M40" s="13"/>
-      <c r="N40" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O40" s="28"/>
-      <c r="P40" s="36"/>
-      <c r="Q40" s="37"/>
+      <c r="N40" s="14"/>
+      <c r="O40" s="26"/>
+      <c r="P40" s="34"/>
+      <c r="Q40" s="35"/>
       <c r="R40" s="18"/>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
@@ -2809,34 +3070,47 @@
       <c r="Y40" s="3"/>
     </row>
     <row r="41" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
+      <c r="B41" s="13">
+        <v>0</v>
+      </c>
+      <c r="C41" s="13">
+        <v>0</v>
+      </c>
+      <c r="D41" s="13">
+        <v>0</v>
+      </c>
       <c r="E41" s="13">
-        <v>1</v>
-      </c>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="F41" s="13">
+        <v>0</v>
+      </c>
+      <c r="G41" s="13">
+        <v>0</v>
+      </c>
+      <c r="H41" s="13">
+        <v>3</v>
+      </c>
       <c r="I41" s="13">
-        <v>1</v>
-      </c>
-      <c r="J41" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="J41" s="13">
+        <v>0</v>
+      </c>
       <c r="K41" s="13">
-        <v>1</v>
-      </c>
-      <c r="L41" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="L41" s="13">
+        <v>0</v>
+      </c>
       <c r="M41" s="13"/>
-      <c r="N41" s="14">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="O41" s="28"/>
-      <c r="P41" s="36"/>
-      <c r="Q41" s="37"/>
+      <c r="N41" s="14"/>
+      <c r="O41" s="26"/>
+      <c r="P41" s="34"/>
+      <c r="Q41" s="35"/>
       <c r="R41" s="18"/>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
@@ -2847,32 +3121,47 @@
       <c r="Y41" s="3"/>
     </row>
     <row r="42" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="33" t="s">
+      <c r="A42" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
+      <c r="B42" s="13">
+        <v>0</v>
+      </c>
+      <c r="C42" s="13">
+        <v>0</v>
+      </c>
+      <c r="D42" s="13">
+        <v>0</v>
+      </c>
       <c r="E42" s="13">
-        <v>1</v>
-      </c>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="F42" s="13">
+        <v>0</v>
+      </c>
+      <c r="G42" s="13">
+        <v>0</v>
+      </c>
+      <c r="H42" s="13">
+        <v>0</v>
+      </c>
+      <c r="I42" s="13">
+        <v>0</v>
+      </c>
+      <c r="J42" s="13">
+        <v>0</v>
+      </c>
       <c r="K42" s="13">
-        <v>5</v>
-      </c>
-      <c r="L42" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="L42" s="13">
+        <v>0</v>
+      </c>
       <c r="M42" s="13"/>
-      <c r="N42" s="14">
-        <f t="shared" si="3"/>
-        <v>6</v>
-      </c>
-      <c r="O42" s="28"/>
-      <c r="P42" s="36"/>
-      <c r="Q42" s="37"/>
+      <c r="N42" s="14"/>
+      <c r="O42" s="26"/>
+      <c r="P42" s="34"/>
+      <c r="Q42" s="35"/>
       <c r="R42" s="18"/>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
@@ -2883,30 +3172,49 @@
       <c r="Y42" s="3"/>
     </row>
     <row r="43" spans="1:25" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="30" t="s">
+      <c r="A43" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
+      <c r="B43" s="13">
+        <v>0</v>
+      </c>
+      <c r="C43" s="13">
+        <v>0</v>
+      </c>
+      <c r="D43" s="13">
+        <v>0</v>
+      </c>
+      <c r="E43" s="13">
+        <v>0</v>
+      </c>
+      <c r="F43" s="13">
+        <v>0</v>
+      </c>
+      <c r="G43" s="13">
+        <v>0</v>
+      </c>
+      <c r="H43" s="13">
+        <v>0</v>
+      </c>
       <c r="I43" s="13">
-        <v>1</v>
-      </c>
-      <c r="J43" s="13"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="13"/>
-      <c r="N43" s="14">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="O43" s="28"/>
-      <c r="P43" s="38"/>
-      <c r="Q43" s="39"/>
+        <v>0</v>
+      </c>
+      <c r="J43" s="13">
+        <v>0</v>
+      </c>
+      <c r="K43" s="13">
+        <v>0</v>
+      </c>
+      <c r="L43" s="13">
+        <v>0</v>
+      </c>
+      <c r="M43" s="13">
+        <v>0</v>
+      </c>
+      <c r="N43" s="14"/>
+      <c r="O43" s="26"/>
+      <c r="P43" s="36"/>
+      <c r="Q43" s="37"/>
       <c r="R43" s="18"/>
       <c r="S43" s="3"/>
       <c r="T43" s="3"/>
@@ -2917,7 +3225,7 @@
       <c r="Y43" s="3"/>
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="N44" s="29"/>
+      <c r="N44" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -2937,4 +3245,13 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>